<commit_message>
Step 2: MLA tab — 7 market leasing assumption rows (property × unit type)
</commit_message>
<xml_diff>
--- a/DFW_Underwriting_Model.xlsx
+++ b/DFW_Underwriting_Model.xlsx
@@ -205,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -239,6 +239,9 @@
     <xf numFmtId="168" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -313,6 +316,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>model</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>MLA data rows 5 to 11</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2280,10 +2298,459 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MARKET LEASING ASSUMPTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Defaults to OM values. Edit per property/unit type to override global assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Property / Unit Type</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>Unit Type</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>Market Rent ($/SF)</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>Rent Growth</t>
+        </is>
+      </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>In-Lease Escalator</t>
+        </is>
+      </c>
+      <c r="F4" s="31" t="inlineStr">
+        <is>
+          <t>Lease Term (mo)</t>
+        </is>
+      </c>
+      <c r="G4" s="31" t="inlineStr">
+        <is>
+          <t>TI New $/SF</t>
+        </is>
+      </c>
+      <c r="H4" s="31" t="inlineStr">
+        <is>
+          <t>TI Renewal $/SF</t>
+        </is>
+      </c>
+      <c r="I4" s="31" t="inlineStr">
+        <is>
+          <t>LC New %</t>
+        </is>
+      </c>
+      <c r="J4" s="31" t="inlineStr">
+        <is>
+          <t>LC Renewal %</t>
+        </is>
+      </c>
+      <c r="K4" s="31" t="inlineStr">
+        <is>
+          <t>Downtime New (mo)</t>
+        </is>
+      </c>
+      <c r="L4" s="31" t="inlineStr">
+        <is>
+          <t>Retention %</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Carrollton — Shop</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D5" s="13">
+        <f>GrowthMarketRent</f>
+        <v/>
+      </c>
+      <c r="E5" s="13">
+        <f>EscalatorInLease</f>
+        <v/>
+      </c>
+      <c r="F5" s="23">
+        <f>LeaseTermMonths</f>
+        <v/>
+      </c>
+      <c r="G5" s="16">
+        <f>TINew</f>
+        <v/>
+      </c>
+      <c r="H5" s="16">
+        <f>TIRenewal</f>
+        <v/>
+      </c>
+      <c r="I5" s="13">
+        <f>LCNew</f>
+        <v/>
+      </c>
+      <c r="J5" s="13">
+        <f>LCRenewal</f>
+        <v/>
+      </c>
+      <c r="K5" s="23">
+        <f>DowntimeNew</f>
+        <v/>
+      </c>
+      <c r="L5" s="13">
+        <f>Retention</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Carrollton — Studio</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Studio</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D6" s="13">
+        <f>GrowthMarketRent</f>
+        <v/>
+      </c>
+      <c r="E6" s="13">
+        <f>EscalatorInLease</f>
+        <v/>
+      </c>
+      <c r="F6" s="23">
+        <f>LeaseTermMonths</f>
+        <v/>
+      </c>
+      <c r="G6" s="16">
+        <f>TINew</f>
+        <v/>
+      </c>
+      <c r="H6" s="16">
+        <f>TIRenewal</f>
+        <v/>
+      </c>
+      <c r="I6" s="13">
+        <f>LCNew</f>
+        <v/>
+      </c>
+      <c r="J6" s="13">
+        <f>LCRenewal</f>
+        <v/>
+      </c>
+      <c r="K6" s="23">
+        <f>DowntimeNew</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>Retention</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Frisco</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D7" s="13">
+        <f>GrowthMarketRent</f>
+        <v/>
+      </c>
+      <c r="E7" s="13">
+        <f>EscalatorInLease</f>
+        <v/>
+      </c>
+      <c r="F7" s="23">
+        <f>LeaseTermMonths</f>
+        <v/>
+      </c>
+      <c r="G7" s="16">
+        <f>TINew</f>
+        <v/>
+      </c>
+      <c r="H7" s="16">
+        <f>TIRenewal</f>
+        <v/>
+      </c>
+      <c r="I7" s="13">
+        <f>LCNew</f>
+        <v/>
+      </c>
+      <c r="J7" s="13">
+        <f>LCRenewal</f>
+        <v/>
+      </c>
+      <c r="K7" s="23">
+        <f>DowntimeNew</f>
+        <v/>
+      </c>
+      <c r="L7" s="13">
+        <f>Retention</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Lewisville</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="D8" s="13">
+        <f>GrowthMarketRent</f>
+        <v/>
+      </c>
+      <c r="E8" s="13">
+        <f>EscalatorInLease</f>
+        <v/>
+      </c>
+      <c r="F8" s="23">
+        <f>LeaseTermMonths</f>
+        <v/>
+      </c>
+      <c r="G8" s="16">
+        <f>TINew</f>
+        <v/>
+      </c>
+      <c r="H8" s="16">
+        <f>TIRenewal</f>
+        <v/>
+      </c>
+      <c r="I8" s="13">
+        <f>LCNew</f>
+        <v/>
+      </c>
+      <c r="J8" s="13">
+        <f>LCRenewal</f>
+        <v/>
+      </c>
+      <c r="K8" s="23">
+        <f>DowntimeNew</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>Retention</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Mesquite</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D9" s="13">
+        <f>GrowthMarketRent</f>
+        <v/>
+      </c>
+      <c r="E9" s="13">
+        <f>EscalatorInLease</f>
+        <v/>
+      </c>
+      <c r="F9" s="23">
+        <f>LeaseTermMonths</f>
+        <v/>
+      </c>
+      <c r="G9" s="16">
+        <f>TINew</f>
+        <v/>
+      </c>
+      <c r="H9" s="16">
+        <f>TIRenewal</f>
+        <v/>
+      </c>
+      <c r="I9" s="13">
+        <f>LCNew</f>
+        <v/>
+      </c>
+      <c r="J9" s="13">
+        <f>LCRenewal</f>
+        <v/>
+      </c>
+      <c r="K9" s="23">
+        <f>DowntimeNew</f>
+        <v/>
+      </c>
+      <c r="L9" s="13">
+        <f>Retention</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Plano</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="D10" s="13">
+        <f>GrowthMarketRent</f>
+        <v/>
+      </c>
+      <c r="E10" s="13">
+        <f>EscalatorInLease</f>
+        <v/>
+      </c>
+      <c r="F10" s="23">
+        <f>LeaseTermMonths</f>
+        <v/>
+      </c>
+      <c r="G10" s="16">
+        <f>TINew</f>
+        <v/>
+      </c>
+      <c r="H10" s="16">
+        <f>TIRenewal</f>
+        <v/>
+      </c>
+      <c r="I10" s="13">
+        <f>LCNew</f>
+        <v/>
+      </c>
+      <c r="J10" s="13">
+        <f>LCRenewal</f>
+        <v/>
+      </c>
+      <c r="K10" s="23">
+        <f>DowntimeNew</f>
+        <v/>
+      </c>
+      <c r="L10" s="13">
+        <f>Retention</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Roanoke</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D11" s="13">
+        <f>GrowthMarketRent</f>
+        <v/>
+      </c>
+      <c r="E11" s="13">
+        <f>EscalatorInLease</f>
+        <v/>
+      </c>
+      <c r="F11" s="23">
+        <f>LeaseTermMonths</f>
+        <v/>
+      </c>
+      <c r="G11" s="16">
+        <f>TINew</f>
+        <v/>
+      </c>
+      <c r="H11" s="16">
+        <f>TIRenewal</f>
+        <v/>
+      </c>
+      <c r="I11" s="13">
+        <f>LCNew</f>
+        <v/>
+      </c>
+      <c r="J11" s="13">
+        <f>LCRenewal</f>
+        <v/>
+      </c>
+      <c r="K11" s="23">
+        <f>DowntimeNew</f>
+        <v/>
+      </c>
+      <c r="L11" s="13">
+        <f>Retention</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>